<commit_message>
feat(users): replace inline user entry fields with a modern popup modal overlay
</commit_message>
<xml_diff>
--- a/Git_hespy.xlsx
+++ b/Git_hespy.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="17">
   <si>
     <t>کلمه کلیدی در کیت هاب</t>
   </si>
@@ -135,12 +135,18 @@
   <si>
     <t>دستور پول از گیتهاب</t>
   </si>
+  <si>
+    <t>«نسخه hespy3 را بازیابی / پول کن»</t>
+  </si>
+  <si>
+    <t>کدینگ سرفصل پیش فرض برای شرکت نمونه نگار بارگذاری شده و کد طوری اصلاح شده که از این به بعد برای هر شرکت جدید کدینگ نمونه بارگذاری خواهد شد</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,6 +170,13 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -185,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +215,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,7 +501,7 @@
   <cols>
     <col min="3" max="3" width="14.42578125" customWidth="1"/>
     <col min="4" max="4" width="56.42578125" customWidth="1"/>
-    <col min="5" max="5" width="30.28515625" customWidth="1"/>
+    <col min="5" max="5" width="34.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -543,7 +557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -554,7 +568,12 @@
         <f t="shared" si="0"/>
         <v>hespy3</v>
       </c>
-      <c r="D4" s="1"/>
+      <c r="D4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">

</xml_diff>

<commit_message>
fix(auth): force fresh login on every app launch - add ?logout=1 param to bat/main.py browser open, clear session in DOMContentLoaded
</commit_message>
<xml_diff>
--- a/Git_hespy.xlsx
+++ b/Git_hespy.xlsx
@@ -12,9 +12,10 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
-    <sheet name="Git_hespy" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="کارهای انجام شده تا کجا" sheetId="4" r:id="rId1"/>
+    <sheet name="Git_hespy" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="نوشتن چند خطی در اکسل" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -69,12 +70,6 @@
       </rPr>
       <t> را بفرمایید، برنامه دقیقاً به همین وضعیت و مرحله با دستور زیر بازگردانی و پول خواهد شد</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">این تست 
-متن چند خطی
-برای ورود به یک سلول اکسل هست
-</t>
   </si>
   <si>
     <t xml:space="preserve">سلام
@@ -140,6 +135,13 @@
   </si>
   <si>
     <t>کدینگ سرفصل پیش فرض برای شرکت نمونه نگار بارگذاری شده و کد طوری اصلاح شده که از این به بعد برای هر شرکت جدید کدینگ نمونه بارگذاری خواهد شد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">این تست 
+متن چند خطی
+برای ورود به یک سلول اکسل هست
+با کلیدهای آلت + اینتر ، در یک سلول جاری نشانگر به خط بعدی می رود
+</t>
   </si>
 </sst>
 </file>
@@ -496,6 +498,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -518,7 +529,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -536,7 +547,7 @@
         <v>5</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -554,7 +565,7 @@
         <v>6</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.3">
@@ -569,10 +580,10 @@
         <v>hespy3</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1829,7 +1840,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:C90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1844,21 +1855,21 @@
         <v>7</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2289,7 +2300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="D5:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2297,14 +2308,14 @@
     <col min="4" max="4" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="4:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:4" ht="120" x14ac:dyDescent="0.25">
       <c r="D5" s="4" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="4:4" ht="45" x14ac:dyDescent="0.25">
       <c r="D7" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hespy5: Milestone release - update database, license state, and milestone records
</commit_message>
<xml_diff>
--- a/Git_hespy.xlsx
+++ b/Git_hespy.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="کارهای انجام شده تا کجا" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="20">
   <si>
     <t>کلمه کلیدی در کیت هاب</t>
   </si>
@@ -143,12 +143,21 @@
 با کلیدهای آلت + اینتر ، در یک سلول جاری نشانگر به خط بعدی می رود
 </t>
   </si>
+  <si>
+    <t>«پروژه را به تگ hespy4 برگردون»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تا مرحله جایگاه ها در انبارها و اختصاص جایگاهها به کالا ها می باشد </t>
+  </si>
+  <si>
+    <t>ورود به برنامه با کد کاربر دیگر کار می کنه ، محدودیت تعداد شرکت برای کاربر میانی کار می کنه</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +188,14 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -200,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -218,6 +235,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,7 +576,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="str">
-        <f t="shared" ref="C3:C66" si="0">CONCATENATE(A3,B3)</f>
+        <f>CONCATENATE(A3,B3)</f>
         <v>hespy2</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -576,7 +594,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A4,B4)</f>
         <v>hespy3</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -594,12 +612,17 @@
         <v>4</v>
       </c>
       <c r="C5" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A5,B5)</f>
         <v>hespy4</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -607,10 +630,12 @@
         <v>5</v>
       </c>
       <c r="C6" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A6,B6)</f>
         <v>hespy5</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
@@ -620,10 +645,11 @@
         <v>6</v>
       </c>
       <c r="C7" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A7,B7)</f>
         <v>hespy6</v>
       </c>
       <c r="D7" s="1"/>
+      <c r="E7" s="7"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -633,7 +659,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A8,B8)</f>
         <v>hespy7</v>
       </c>
       <c r="D8" s="1"/>
@@ -646,7 +672,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A9,B9)</f>
         <v>hespy8</v>
       </c>
       <c r="D9" s="1"/>
@@ -659,7 +685,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A10,B10)</f>
         <v>hespy9</v>
       </c>
       <c r="D10" s="1"/>
@@ -672,7 +698,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A11,B11)</f>
         <v>hespy10</v>
       </c>
       <c r="D11" s="1"/>
@@ -685,7 +711,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A12,B12)</f>
         <v>hespy11</v>
       </c>
       <c r="D12" s="1"/>
@@ -698,7 +724,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A13,B13)</f>
         <v>hespy12</v>
       </c>
       <c r="D13" s="1"/>
@@ -711,7 +737,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A14,B14)</f>
         <v>hespy13</v>
       </c>
       <c r="D14" s="1"/>
@@ -724,7 +750,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A15,B15)</f>
         <v>hespy14</v>
       </c>
       <c r="D15" s="1"/>
@@ -737,7 +763,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A16,B16)</f>
         <v>hespy15</v>
       </c>
       <c r="D16" s="1"/>
@@ -750,7 +776,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A17,B17)</f>
         <v>hespy16</v>
       </c>
       <c r="D17" s="1"/>
@@ -763,7 +789,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A18,B18)</f>
         <v>hespy17</v>
       </c>
       <c r="D18" s="1"/>
@@ -776,7 +802,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A19,B19)</f>
         <v>hespy18</v>
       </c>
       <c r="D19" s="1"/>
@@ -789,7 +815,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A20,B20)</f>
         <v>hespy19</v>
       </c>
       <c r="D20" s="1"/>
@@ -802,7 +828,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A21,B21)</f>
         <v>hespy20</v>
       </c>
       <c r="D21" s="1"/>
@@ -815,7 +841,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A22,B22)</f>
         <v>hespy21</v>
       </c>
       <c r="D22" s="1"/>
@@ -828,7 +854,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A23,B23)</f>
         <v>hespy22</v>
       </c>
       <c r="D23" s="1"/>
@@ -841,7 +867,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A24,B24)</f>
         <v>hespy23</v>
       </c>
       <c r="D24" s="1"/>
@@ -854,7 +880,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A25,B25)</f>
         <v>hespy24</v>
       </c>
       <c r="D25" s="1"/>
@@ -867,7 +893,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A26,B26)</f>
         <v>hespy25</v>
       </c>
       <c r="D26" s="1"/>
@@ -880,7 +906,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A27,B27)</f>
         <v>hespy26</v>
       </c>
       <c r="D27" s="1"/>
@@ -893,7 +919,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A28,B28)</f>
         <v>hespy27</v>
       </c>
       <c r="D28" s="1"/>
@@ -906,7 +932,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A29,B29)</f>
         <v>hespy28</v>
       </c>
       <c r="D29" s="1"/>
@@ -919,7 +945,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A30,B30)</f>
         <v>hespy29</v>
       </c>
       <c r="D30" s="1"/>
@@ -932,7 +958,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A31,B31)</f>
         <v>hespy30</v>
       </c>
       <c r="D31" s="1"/>
@@ -945,7 +971,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A32,B32)</f>
         <v>hespy31</v>
       </c>
       <c r="D32" s="1"/>
@@ -958,7 +984,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A33,B33)</f>
         <v>hespy32</v>
       </c>
       <c r="D33" s="1"/>
@@ -971,7 +997,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A34,B34)</f>
         <v>hespy33</v>
       </c>
       <c r="D34" s="1"/>
@@ -984,7 +1010,7 @@
         <v>34</v>
       </c>
       <c r="C35" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A35,B35)</f>
         <v>hespy34</v>
       </c>
       <c r="D35" s="1"/>
@@ -997,7 +1023,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A36,B36)</f>
         <v>hespy35</v>
       </c>
       <c r="D36" s="1"/>
@@ -1010,7 +1036,7 @@
         <v>36</v>
       </c>
       <c r="C37" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A37,B37)</f>
         <v>hespy36</v>
       </c>
       <c r="D37" s="1"/>
@@ -1023,7 +1049,7 @@
         <v>37</v>
       </c>
       <c r="C38" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A38,B38)</f>
         <v>hespy37</v>
       </c>
       <c r="D38" s="1"/>
@@ -1036,7 +1062,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A39,B39)</f>
         <v>hespy38</v>
       </c>
       <c r="D39" s="1"/>
@@ -1049,7 +1075,7 @@
         <v>39</v>
       </c>
       <c r="C40" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A40,B40)</f>
         <v>hespy39</v>
       </c>
       <c r="D40" s="1"/>
@@ -1062,7 +1088,7 @@
         <v>40</v>
       </c>
       <c r="C41" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A41,B41)</f>
         <v>hespy40</v>
       </c>
       <c r="D41" s="1"/>
@@ -1075,7 +1101,7 @@
         <v>41</v>
       </c>
       <c r="C42" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A42,B42)</f>
         <v>hespy41</v>
       </c>
       <c r="D42" s="1"/>
@@ -1088,7 +1114,7 @@
         <v>42</v>
       </c>
       <c r="C43" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A43,B43)</f>
         <v>hespy42</v>
       </c>
       <c r="D43" s="1"/>
@@ -1101,7 +1127,7 @@
         <v>43</v>
       </c>
       <c r="C44" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A44,B44)</f>
         <v>hespy43</v>
       </c>
       <c r="D44" s="1"/>
@@ -1114,7 +1140,7 @@
         <v>44</v>
       </c>
       <c r="C45" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A45,B45)</f>
         <v>hespy44</v>
       </c>
       <c r="D45" s="1"/>
@@ -1127,7 +1153,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A46,B46)</f>
         <v>hespy45</v>
       </c>
       <c r="D46" s="1"/>
@@ -1140,7 +1166,7 @@
         <v>46</v>
       </c>
       <c r="C47" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A47,B47)</f>
         <v>hespy46</v>
       </c>
       <c r="D47" s="1"/>
@@ -1153,7 +1179,7 @@
         <v>47</v>
       </c>
       <c r="C48" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A48,B48)</f>
         <v>hespy47</v>
       </c>
       <c r="D48" s="1"/>
@@ -1166,7 +1192,7 @@
         <v>48</v>
       </c>
       <c r="C49" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A49,B49)</f>
         <v>hespy48</v>
       </c>
       <c r="D49" s="1"/>
@@ -1179,7 +1205,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A50,B50)</f>
         <v>hespy49</v>
       </c>
       <c r="D50" s="1"/>
@@ -1192,7 +1218,7 @@
         <v>50</v>
       </c>
       <c r="C51" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A51,B51)</f>
         <v>hespy50</v>
       </c>
       <c r="D51" s="1"/>
@@ -1205,7 +1231,7 @@
         <v>51</v>
       </c>
       <c r="C52" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A52,B52)</f>
         <v>hespy51</v>
       </c>
       <c r="D52" s="1"/>
@@ -1218,7 +1244,7 @@
         <v>52</v>
       </c>
       <c r="C53" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A53,B53)</f>
         <v>hespy52</v>
       </c>
       <c r="D53" s="1"/>
@@ -1231,7 +1257,7 @@
         <v>53</v>
       </c>
       <c r="C54" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A54,B54)</f>
         <v>hespy53</v>
       </c>
       <c r="D54" s="1"/>
@@ -1244,7 +1270,7 @@
         <v>54</v>
       </c>
       <c r="C55" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A55,B55)</f>
         <v>hespy54</v>
       </c>
       <c r="D55" s="1"/>
@@ -1257,7 +1283,7 @@
         <v>55</v>
       </c>
       <c r="C56" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A56,B56)</f>
         <v>hespy55</v>
       </c>
       <c r="D56" s="1"/>
@@ -1270,7 +1296,7 @@
         <v>56</v>
       </c>
       <c r="C57" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A57,B57)</f>
         <v>hespy56</v>
       </c>
       <c r="D57" s="1"/>
@@ -1283,7 +1309,7 @@
         <v>57</v>
       </c>
       <c r="C58" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A58,B58)</f>
         <v>hespy57</v>
       </c>
       <c r="D58" s="1"/>
@@ -1296,7 +1322,7 @@
         <v>58</v>
       </c>
       <c r="C59" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A59,B59)</f>
         <v>hespy58</v>
       </c>
       <c r="D59" s="1"/>
@@ -1309,7 +1335,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A60,B60)</f>
         <v>hespy59</v>
       </c>
       <c r="D60" s="1"/>
@@ -1322,7 +1348,7 @@
         <v>60</v>
       </c>
       <c r="C61" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A61,B61)</f>
         <v>hespy60</v>
       </c>
       <c r="D61" s="1"/>
@@ -1335,7 +1361,7 @@
         <v>61</v>
       </c>
       <c r="C62" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A62,B62)</f>
         <v>hespy61</v>
       </c>
       <c r="D62" s="1"/>
@@ -1348,7 +1374,7 @@
         <v>62</v>
       </c>
       <c r="C63" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A63,B63)</f>
         <v>hespy62</v>
       </c>
       <c r="D63" s="1"/>
@@ -1361,7 +1387,7 @@
         <v>63</v>
       </c>
       <c r="C64" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A64,B64)</f>
         <v>hespy63</v>
       </c>
       <c r="D64" s="1"/>
@@ -1374,7 +1400,7 @@
         <v>64</v>
       </c>
       <c r="C65" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A65,B65)</f>
         <v>hespy64</v>
       </c>
       <c r="D65" s="1"/>
@@ -1387,7 +1413,7 @@
         <v>65</v>
       </c>
       <c r="C66" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>CONCATENATE(A66,B66)</f>
         <v>hespy65</v>
       </c>
       <c r="D66" s="1"/>
@@ -1400,7 +1426,7 @@
         <v>66</v>
       </c>
       <c r="C67" s="2" t="str">
-        <f t="shared" ref="C67:C100" si="1">CONCATENATE(A67,B67)</f>
+        <f>CONCATENATE(A67,B67)</f>
         <v>hespy66</v>
       </c>
       <c r="D67" s="1"/>
@@ -1413,7 +1439,7 @@
         <v>67</v>
       </c>
       <c r="C68" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A68,B68)</f>
         <v>hespy67</v>
       </c>
       <c r="D68" s="1"/>
@@ -1426,7 +1452,7 @@
         <v>68</v>
       </c>
       <c r="C69" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A69,B69)</f>
         <v>hespy68</v>
       </c>
       <c r="D69" s="1"/>
@@ -1439,7 +1465,7 @@
         <v>69</v>
       </c>
       <c r="C70" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A70,B70)</f>
         <v>hespy69</v>
       </c>
       <c r="D70" s="1"/>
@@ -1452,7 +1478,7 @@
         <v>70</v>
       </c>
       <c r="C71" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A71,B71)</f>
         <v>hespy70</v>
       </c>
       <c r="D71" s="1"/>
@@ -1465,7 +1491,7 @@
         <v>71</v>
       </c>
       <c r="C72" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A72,B72)</f>
         <v>hespy71</v>
       </c>
       <c r="D72" s="1"/>
@@ -1478,7 +1504,7 @@
         <v>72</v>
       </c>
       <c r="C73" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A73,B73)</f>
         <v>hespy72</v>
       </c>
       <c r="D73" s="1"/>
@@ -1491,7 +1517,7 @@
         <v>73</v>
       </c>
       <c r="C74" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A74,B74)</f>
         <v>hespy73</v>
       </c>
       <c r="D74" s="1"/>
@@ -1504,7 +1530,7 @@
         <v>74</v>
       </c>
       <c r="C75" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A75,B75)</f>
         <v>hespy74</v>
       </c>
       <c r="D75" s="1"/>
@@ -1517,7 +1543,7 @@
         <v>75</v>
       </c>
       <c r="C76" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A76,B76)</f>
         <v>hespy75</v>
       </c>
       <c r="D76" s="1"/>
@@ -1530,7 +1556,7 @@
         <v>76</v>
       </c>
       <c r="C77" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A77,B77)</f>
         <v>hespy76</v>
       </c>
       <c r="D77" s="1"/>
@@ -1543,7 +1569,7 @@
         <v>77</v>
       </c>
       <c r="C78" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A78,B78)</f>
         <v>hespy77</v>
       </c>
       <c r="D78" s="1"/>
@@ -1556,7 +1582,7 @@
         <v>78</v>
       </c>
       <c r="C79" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A79,B79)</f>
         <v>hespy78</v>
       </c>
       <c r="D79" s="1"/>
@@ -1569,7 +1595,7 @@
         <v>79</v>
       </c>
       <c r="C80" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A80,B80)</f>
         <v>hespy79</v>
       </c>
       <c r="D80" s="1"/>
@@ -1582,7 +1608,7 @@
         <v>80</v>
       </c>
       <c r="C81" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A81,B81)</f>
         <v>hespy80</v>
       </c>
       <c r="D81" s="1"/>
@@ -1595,7 +1621,7 @@
         <v>81</v>
       </c>
       <c r="C82" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A82,B82)</f>
         <v>hespy81</v>
       </c>
       <c r="D82" s="1"/>
@@ -1608,7 +1634,7 @@
         <v>82</v>
       </c>
       <c r="C83" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A83,B83)</f>
         <v>hespy82</v>
       </c>
       <c r="D83" s="1"/>
@@ -1621,7 +1647,7 @@
         <v>83</v>
       </c>
       <c r="C84" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A84,B84)</f>
         <v>hespy83</v>
       </c>
       <c r="D84" s="1"/>
@@ -1634,7 +1660,7 @@
         <v>84</v>
       </c>
       <c r="C85" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A85,B85)</f>
         <v>hespy84</v>
       </c>
       <c r="D85" s="1"/>
@@ -1647,7 +1673,7 @@
         <v>85</v>
       </c>
       <c r="C86" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A86,B86)</f>
         <v>hespy85</v>
       </c>
       <c r="D86" s="1"/>
@@ -1660,7 +1686,7 @@
         <v>86</v>
       </c>
       <c r="C87" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A87,B87)</f>
         <v>hespy86</v>
       </c>
       <c r="D87" s="1"/>
@@ -1673,7 +1699,7 @@
         <v>87</v>
       </c>
       <c r="C88" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A88,B88)</f>
         <v>hespy87</v>
       </c>
       <c r="D88" s="1"/>
@@ -1686,7 +1712,7 @@
         <v>88</v>
       </c>
       <c r="C89" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A89,B89)</f>
         <v>hespy88</v>
       </c>
       <c r="D89" s="1"/>
@@ -1699,7 +1725,7 @@
         <v>89</v>
       </c>
       <c r="C90" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A90,B90)</f>
         <v>hespy89</v>
       </c>
       <c r="D90" s="1"/>
@@ -1712,7 +1738,7 @@
         <v>90</v>
       </c>
       <c r="C91" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A91,B91)</f>
         <v>hespy90</v>
       </c>
       <c r="D91" s="1"/>
@@ -1725,7 +1751,7 @@
         <v>91</v>
       </c>
       <c r="C92" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A92,B92)</f>
         <v>hespy91</v>
       </c>
       <c r="D92" s="1"/>
@@ -1738,7 +1764,7 @@
         <v>92</v>
       </c>
       <c r="C93" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A93,B93)</f>
         <v>hespy92</v>
       </c>
       <c r="D93" s="1"/>
@@ -1751,7 +1777,7 @@
         <v>93</v>
       </c>
       <c r="C94" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A94,B94)</f>
         <v>hespy93</v>
       </c>
       <c r="D94" s="1"/>
@@ -1764,7 +1790,7 @@
         <v>94</v>
       </c>
       <c r="C95" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A95,B95)</f>
         <v>hespy94</v>
       </c>
       <c r="D95" s="1"/>
@@ -1777,7 +1803,7 @@
         <v>95</v>
       </c>
       <c r="C96" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A96,B96)</f>
         <v>hespy95</v>
       </c>
       <c r="D96" s="1"/>
@@ -1790,7 +1816,7 @@
         <v>96</v>
       </c>
       <c r="C97" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A97,B97)</f>
         <v>hespy96</v>
       </c>
       <c r="D97" s="1"/>
@@ -1803,7 +1829,7 @@
         <v>97</v>
       </c>
       <c r="C98" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A98,B98)</f>
         <v>hespy97</v>
       </c>
       <c r="D98" s="1"/>
@@ -1816,7 +1842,7 @@
         <v>98</v>
       </c>
       <c r="C99" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A99,B99)</f>
         <v>hespy98</v>
       </c>
       <c r="D99" s="1"/>
@@ -1829,7 +1855,7 @@
         <v>99</v>
       </c>
       <c r="C100" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE(A100,B100)</f>
         <v>hespy99</v>
       </c>
       <c r="D100" s="1"/>

</xml_diff>

<commit_message>
hespy6: Update milestone document Git_hespy.xlsx
</commit_message>
<xml_diff>
--- a/Git_hespy.xlsx
+++ b/Git_hespy.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="21">
   <si>
     <t>کلمه کلیدی در کیت هاب</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>ورود به برنامه با کد کاربر دیگر کار می کنه ، محدودیت تعداد شرکت برای کاربر میانی کار می کنه</t>
+  </si>
+  <si>
+    <t>ورود به برنامه با کد کاربر دیگر کار می کنه ، محدودیت تعداد شرکت برای کاربر میانی کار می کنه و همچنین محدودیت تعداد سال مالی برای هر شرکت هم اضافه شده است</t>
   </si>
 </sst>
 </file>
@@ -651,7 +654,7 @@
       <c r="D7" s="1"/>
       <c r="E7" s="7"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
@@ -662,7 +665,9 @@
         <f>CONCATENATE(A8,B8)</f>
         <v>hespy7</v>
       </c>
-      <c r="D8" s="1"/>
+      <c r="D8" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">

</xml_diff>

<commit_message>
Negar_Web_PY: Update akharin taghirate code va edame_kar
</commit_message>
<xml_diff>
--- a/Git_hespy.xlsx
+++ b/Git_hespy.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="کارهای انجام شده تا کجا" sheetId="4" r:id="rId1"/>
@@ -2333,20 +2333,37 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="D5:D7"/>
+  <dimension ref="D5:N7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="38.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="4:4" ht="120" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:14" ht="120" x14ac:dyDescent="0.25">
       <c r="D5" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="4:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:14" ht="45" x14ac:dyDescent="0.25">
       <c r="D7" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="J7">
+        <v>40</v>
+      </c>
+      <c r="K7">
+        <v>20</v>
+      </c>
+      <c r="L7">
+        <f>J7*K7</f>
+        <v>800</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+      <c r="N7">
+        <f>L7*M7</f>
+        <v>8000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>